<commit_message>
Informe DIA EP inicio 2026: nueva seccion Ranking por Nucleo
Agrega al visor la seccion Ranking De Establecimientos Por Nucleo
(solicitud equipo Educacion Parvularia, Estrategia Lenguaje Verbal):
ranking por nucleo con orden por Comenzando o Profundizando,
matricula reportada NT1+NT2 y rubricas efectivamente aplicadas por
establecimiento. Lenguaje verbal como vista por defecto. Incluye
panel interactivo, tabla completa y Excel descargable en assets.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_DIA_inicio_2026_analisis_assets/matriz_global_rubricas.xlsx
+++ b/02_DIA_inicio_2026_analisis_assets/matriz_global_rubricas.xlsx
@@ -2194,13 +2194,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4A4BB135-F861-4D57-950E-B47CE5DB0697}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{79D2A957-00C9-4EED-8902-4DBB29119A0E}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{788091DC-B345-43B0-9E17-E121626780CE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8A0A0FB0-91DF-4D87-B467-4C751BB72D1D}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2707C68-C6A3-4D14-9E8E-15460AF2ABE6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEBADF06-DFA7-4085-A628-1C330F8C5FD4}"/>
 </file>
</xml_diff>